<commit_message>
chore(specsmd): admin-factory-email intent and run artifacts
Also refreshes the requirements traceability matrix and adds the plain-TH
evaluation summary.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/requirements-traceability.xlsx
+++ b/docs/requirements-traceability.xlsx
@@ -14,6 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="009 standard-files" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="010 file-deletion" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="011 reward-guard" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCF score-change-finality" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AFE admin-factory-email" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'003 evaluator-review'!$A$4:$C$14</definedName>
@@ -22,6 +24,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'009 standard-files'!$A$4:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'010 file-deletion'!$A$4:$C$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'011 reward-guard'!$A$4:$C$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'SCF score-change-finality'!$A$4:$C$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'AFE admin-factory-email'!$A$4:$C$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -72,7 +76,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -86,7 +90,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDF2F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -101,17 +120,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
+        <fgColor rgb="00DEEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DEEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -141,10 +155,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -154,36 +170,56 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,16 +587,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -570,10 +606,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TWHP-RTM-EVAL-001 · ข้อมูล ณ 17 สิงหาคม 2569 · ข้อกำหนด 37 ข้อ จาก 6 intent · ผลการทดสอบที่อ้างถึงเป็นผลของวันที่ระบุไว้ ยังไม่ได้รันซ้ำ</t>
+          <t>TWHP-RTM-EVAL-003 · ปรับข้อมูล 26 สิงหาคม 2569 · โมดูลการประเมิน 43 ข้อ จาก 7 intent · เครื่องหมาย ⟲ คือข้อที่ถูก ADR-0012 กลับคำ · ★ คือ intent ล่าสุด · ⚠️ ตัวเลขชุดทดสอบเต็ม 537/0 ของ run 005–010 มาจากทรีที่รวมงาน fiscal-year ไว้ด้วย สาขา dev ปัจจุบันไม่มีงานนั้น (ค้างอยู่ที่ feat/fiscal-year) ชุดทดสอบเต็มบน dev ตอนนี้คือ 392/0 — ตัวเลขรายชุดของโมดูลการประเมินยังตรงกับโค้ดปัจจุบันทุกไฟล์</t>
         </is>
       </c>
     </row>
@@ -614,7 +650,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>003 — การตรวจ Cover แบบลำดับชั้น</t>
@@ -624,24 +660,24 @@
         <v>10</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>งานรุ่นแรก สร้างตอนยังไม่มี test runner จึงมีช่องว่างมากที่สุด</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>⟲ ถูก ADR-0012 ปรับ 6 ข้อ · FR-6 ได้เทสต์แล้ว เหลือ FR-8 ที่ยังใช้การอ่านโค้ด</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>004 — ผู้ดูแลในฐานะ ODPC</t>
@@ -664,11 +700,11 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>ตรรกะใช้ร่วมกับ ODPC จุดอ่อนอยู่ที่ guard และการบันทึกผู้กระทำ (G-1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
+          <t>ไม่มีการเปลี่ยนแปลงรอบนี้ · G-1 ยังเปิดอยู่และยังเป็นจุดที่ควรแก้ก่อน</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>008 — การตรวจแบบสองเฟส</t>
@@ -691,11 +727,11 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>ครบทุกข้อ เป็นแกนที่แข็งแรงที่สุดของโมดูล</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+          <t>⟲ FR-2, FR-3, FR-6 ปรับตาม ADR-0012 · ยังครบทุกข้อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>009 — ไฟล์มาตรฐาน</t>
@@ -718,38 +754,38 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>ครบทุกข้อ เหลือแค่เรื่อง N+1 ที่ยืนยันด้วยการอ่านโค้ด</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>ข้อมูลชุดนี้ถูกต่อยอดไปใช้ตอน hard reject ใน SCF-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>010 — ลบไฟล์เมื่อปรับคะแนน</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="5" t="n">
+      <c r="C9" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>ครบทุกข้อ เทสต์เดิมรองรับอยู่แล้วเกือบทั้งหมด</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
+      <c r="F9" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>⚠️ ถูกกลับคำเกือบทั้ง intent — ADR-0006 ถูกแทนที่ทั้งฉบับ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>011 — Grade เฉพาะ Cover ที่เสร็จ</t>
@@ -759,10 +795,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>0</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>5</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>0</v>
@@ -772,217 +808,365 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>เขียนเทสต์ครบแล้วแต่ยังไม่ได้รัน เป็นงานค้าง (G-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+          <t>✓ commit แล้วและอยู่ในชุดทดสอบเต็มที่ผ่าน — ปิดช่องว่าง G-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="32" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>SCF — Score-Change Finality ★</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>intent ล่าสุด ปิดงาน 25 ส.ค. 2569 · 6 work item · run 005–010 · ครบทุกข้อ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>รวม</t>
         </is>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>37</v>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>28</v>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว 76% · ไม่มีข้อไหนที่ไม่ได้ตรวจเลย</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="B12" s="10" t="n">
+        <v>43</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว 88% · ไม่มีข้อไหนที่ไม่ได้ตรวจเลย · ไม่เหลือข้อที่เขียนเทสต์แล้วแต่ยังไม่ได้รัน</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>AFE — Admin Factory List (นอกขอบเขต) ⚑</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>run 011 · 26 ส.ค. 2569 · เป็นงานโดเมนโรงงาน ไม่ได้นับรวมในยอด 43 ข้อข้างบน · ยังไม่ commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>ช่องว่างที่เจอจากการจับคู่</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>รหัส</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>ข้อกำหนด</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>สถานะ</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>ช่องว่าง</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>เกี่ยวข้องกับ</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="64" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>หมายเหตุ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>G-1</t>
         </is>
       </c>
-      <c r="B15" s="11" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>004-FR-6</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>การตรวจว่าใครเป็นคนทำฝั่งผู้ดูแลหายไป — bolt 012 เคยตรวจไว้ แต่ bolt 021 เอาไฟล์ทดสอบอื่นมาทับ ตอนนี้ไม่มีกรณีไหนตรวจว่าการสรุปผลโดยผู้ดูแล เขียน id ลง coverLogs.evaluatorId เป็นข้อเดียวที่ความครอบคลุมถอยหลัง</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>ใหม่ — ควรแก้ก่อนใคร</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>เปิดอยู่</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>การตรวจว่าใครเป็นคนทำฝั่งผู้ดูแลหายไป — bolt 012 เคยตรวจไว้ แต่ bolt 021 เอาไฟล์ทดสอบอื่นมาทับ ตอนนี้ไม่มีกรณีไหนตรวจว่าการสรุปผลโดยผู้ดูแลเขียน id ลง coverLogs.evaluatorId งานของ intent ล่าสุดไม่ได้แตะจุดนี้ จึงยังเป็นข้อเดียวที่ความครอบคลุมถอยหลัง</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>ควรแก้ก่อนใคร</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="52" customHeight="1">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>G-2</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>003-FR-6, 003-FR-8</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>วงจรต่อรองและเงื่อนไขการส่งซ้ำยังใช้การอ่านโค้ดจาก bolt 009 เป็นพื้นที่ที่ยังใช้งานจริงและใหญ่ที่สุดที่ไม่มีกรณีทดสอบ</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>003-FR-8</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>แคบลง</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>เดิมครอบคลุมทั้งวงจรต่อรองและเงื่อนไขการส่งซ้ำ ตอนนี้ run 007 เขียนเทสต์ให้ negotiate แล้ว เหลือแค่เงื่อนไขการส่งซ้ำที่ยังใช้การอ่านโค้ดจาก bolt 009 อยู่ข้อเดียว</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>test-report หัวข้อ 9</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="19" ht="52" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>G-3</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>003-FR-9</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>ตอนสรุปผลตรวจแค่ว่า Grade อยู่ในชุดค่าที่ถูกต้อง ยังไม่ได้เทียบกับค่าที่ควรได้จากข้อมูลตั้งต้นที่รู้คำตอบแน่นอน</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>เปิดอยู่</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>ตอนสรุปผลตรวจแค่ว่า Grade อยู่ในชุดค่าที่ถูกต้อง ยังไม่ได้เทียบกับค่าที่ควรได้จากข้อมูลตั้งต้น ที่รู้คำตอบแน่นอน แม้ run 006 จะพิสูจน์เพิ่มแล้วว่า Grade ขยับตามคะแนนที่แก้</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>test-report หัวข้อ 9</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>G-4</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>009-FR-4</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>เปิดอยู่</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>ข้อกำหนดไม่เกิด N+1 ยังไม่มีการทดสอบที่นับจำนวนคำสั่งค้นหา</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>G-5</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B21" s="20" t="inlineStr">
         <is>
           <t>011-FR-1…FR-5</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>ทั้ง intent เขียนกรณีทดสอบไว้แล้ว แต่ยังไม่ได้รัน และ bolt 024 ก็ยังไม่มีรายงานผลการทดสอบ</t>
-        </is>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>D-07</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
+        <is>
+          <t>ปิดแล้ว ✓</t>
+        </is>
+      </c>
+      <c r="D21" s="20" t="inlineStr">
+        <is>
+          <t>งานถูก commit และอยู่ในชุดทดสอบเต็มที่ผ่าน 537/0 แล้ว เหลือเพียงข้อสังเกตว่า bolt 024 ยังไม่มีไฟล์รายงานผลการทดสอบของตัวเอง</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="inlineStr">
+        <is>
+          <t>ปิดโดย run 009/010</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="52" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>G-6</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>003-FR-4</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>ข้อกำหนดคะแนนที่ยอมรับกลายเป็นคำตอบที่ใช้จริง ทำงานผ่าน answer.negotiate ซึ่งไม่มีกรณีทดสอบ</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>G-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
+        <is>
+          <t>ปิดแล้ว ✓</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="inlineStr">
+        <is>
+          <t>เดิมคะแนนที่ยอมรับกลายเป็นคำตอบที่ใช้จริงผ่าน answer.negotiate ซึ่งไม่มีเทสต์ ตอนนี้การเขียนค่าย้ายไปอยู่ที่ finalize และมีเทสต์ตรงตัวใน run 006 แล้ว</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>ปิดโดย SCF-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="18" t="inlineStr">
         <is>
           <t>G-7</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>004-FR-3, 008-FR-7</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>เปิดอยู่</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>ทั้งสองฝั่งยืนยันแล้วในระดับ service แต่เส้นทางการปฏิเสธของ adminGuard ยังไม่มีการตรวจ</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>D-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="66" customHeight="1">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>G-8</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>SCF-2</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>ใหม่ · เปิดโดยตั้งใจ</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>หลังสรุปผลแล้ว โรงงานดูคะแนนเดิมที่ตัวเองกรอกไว้ไม่ได้อีก เพราะ selectedChoice ถูกเขียนทับ และไม่มีที่ไหนเก็บค่าเดิมไว้ ยอมรับไว้ตั้งแต่ตอน checkpoint ของ SCF-2 การแก้ต้องเปลี่ยนโครงสร้างฐานข้อมูล จึงแยกเป็น intent ต่างหาก บันทึกไว้ใน ADR-0012 แล้ว</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>run 008 · ต้องแก้ schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="21" t="inlineStr">
+        <is>
+          <t>G-9</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>SCF ทั้ง intent</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>ใหม่ · เลื่อนไว้</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>ยังไม่ได้ backfill แถวเดิมบน production และยังไม่ได้วัดว่ามีกี่แถว (เงื่อนไข verdict_choice IS NULL น่าจะทำให้เหลือเกือบศูนย์ แต่ยังไม่มีตัวเลขจริง) ส่วน Cover ที่ finished ไปแล้วและเสียหลักฐานไปตอน ADR-0006 กู้คืนไม่ได้ เว้นแต่ MinIO เปิด versioning ไว้ ซึ่งควรเช็กก่อนไปแตะ bucket</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
+        <is>
+          <t>ตัดออกจากขอบเขตโดยตั้งใจ · ค้างแจ้ง PO</t>
         </is>
       </c>
     </row>
@@ -1001,8 +1185,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1012,32 +1196,32 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>intent ตั้งต้นที่วางโครงทั้งโมดูล สร้างช่วง bolt 006–010 ซึ่งตอนนั้นยังไม่มี test runner เทสต์ที่รองรับอยู่ทุกวันนี้มาจากงานรุ่นหลังที่ย้อนกลับมาเขียนทับให้</t>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>intent ตั้งต้นที่วางโครงทั้งโมดูล สร้างช่วง bolt 006–010 ซึ่งตอนนั้นยังไม่มี test runner ต่อมาถูก ADR-0012 (25 ส.ค. 2569) กลับคำหลายข้อ โดยเฉพาะเรื่อง change-score และวงจรต่อรอง</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>003-FR-1
 รายการคำตอบตามระดับสิทธิ์</t>
@@ -1048,16 +1232,16 @@
           <t>GET …/covers/:id/answers คืนคำตอบพร้อมสถานะ หมวดคำถาม คำตอบของโรงงาน และคำวินิจฉัยล่าสุด โดยกรองหมวดตามระดับผู้ประเมินที่ฝั่งเซิร์ฟเวอร์ (Mental → Mental ; DOH → Disease + Safety ; ODPC → ครบ 5 หมวด) และจำกัดตามเขตสุขภาพ</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: evaluator-review.integration — กรณีกรองหมวด และผิดเขต 404 ; ขยายเพิ่มโดย intent 009
-ผลที่บันทึกไว้: 50/50, bolt 022, 3 ก.ค. 2569</t>
+ผลที่บันทึกไว้: 10/10 ในชุดนี้ · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>003-FR-2
 บันทึกผลตรวจแบบชุด</t>
@@ -1068,7 +1252,7 @@
           <t>ส่งคำวินิจฉัยหลายข้อพร้อมกันในทรานแซกชันเดียว ถ้ามีข้อไหนอยู่นอกหมวดที่ตัวเองดูแล ให้ปฏิเสธทั้งชุดด้วย 403 โดยไม่บันทึกอะไรเลย</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>เลิกใช้แล้ว
 หลักฐาน: ตรวจด้วยการอ่านโค้ด (bolt 007) ต่อมาเส้นทางถูกลบใน bolt 021 การยิงคำขอได้ผล 404
@@ -1076,51 +1260,53 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="7" ht="94" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>003-FR-3
-คำวินิจฉัย 3 แบบ</t>
+คำวินิจฉัย 3 แบบ  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>approve, change-score (ต้องมีคะแนนเสนอ 0–3 + คำอธิบาย เก็บไฟล์ไว้) และ reject (ไม่มีคะแนนเสนอ + คำอธิบาย ลบไฟล์) พร้อมเพิ่มค่า recommended เข้า answerStatus</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — กรณีผลลัพธ์ของ approve / change_score / reject (ส่วน approve ถูกแก้โดย 008-FR-2)
-ผลที่บันทึกไว้: 19/19, bolt 019, 2 ก.ค. 2569</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="78" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+          <t>เดิม: approve, change-score และ reject ต่างก็ให้ผลของตัวเอง โดย change-score กับ reject ใช้สถานะ rejected ร่วมกัน แยกกันที่ verdict_choice
+⟲ ADR-0012 แยกสองอย่างนี้ออกจากกัน — change-score ได้ recommended พร้อมเก็บ verdictChoice และคำอธิบายไว้ ส่วน reject เท่านั้นที่ได้ rejected ตอนนี้ค่าที่จำแนกคือ status = rejected AND verdict_choice IS NULL</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — change_score → recommended พร้อม verdictChoice + description ที่ยังอยู่ครบ ; reject → rejected + verdictChoice เป็น null ; approve ไม่เปลี่ยน
+ผลที่บันทึกไว้: 26/26, run 005, 24 ส.ค. 2569 (ชุดนี้โต 19 → 26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="94" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>003-FR-4
-คะแนนที่ผู้ประเมินเสนอ</t>
+คะแนนที่ผู้ประเมินเสนอ  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>เก็บใน verdict_choice ได้แค่ 0–3 ห้ามเป็น n/a และห้ามเขียนทับ selectedChoice ของโรงงาน คำตอบที่ใช้คิดคะแนนคือค่าที่ตกลงกันล่าสุด คำวินิจฉัยที่ยังไม่ถูกยอมรับจะไม่กระทบคะแนน</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>ยืนยันบางส่วน
-หลักฐาน: save — เขียน verdict_choice ตอน change_score และ union 0–3 กัน n/a ; answer.integration — การเสริมข้อมูลจากล็อกล่าสุด ส่วนขา “คะแนนที่ยอมรับกลายเป็นคำตอบที่ใช้จริง” อยู่ใน negotiate ซึ่งยังไม่มีเทสต์ (G-6)
-ผลที่บันทึกไว้: 19/19 + 3/3, bolt 019 / 023</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+          <t>เก็บใน verdict_choice ได้แค่ 0–3 ห้ามเป็น n/a
+⟲ ADR-0012 กลับคำข้อ “ห้ามเขียนทับ selectedChoice” — ตอนสรุปผล ระบบจะเขียน verdictChoice ลง answers.selectedChoice ในทรานแซกชันเดียวกับการเลื่อนสถานะ เพื่อให้ Grade คิดจากคะแนนที่ผู้ตรวจแก้จริง ไม่ใช่ค่าเดิมของโรงงาน (เดิมมีแค่ accept ของโรงงานที่เขียนค่านี้ พอเลิกใช้วงจรต่อรองแล้ว การแก้คะแนนจะไม่ถึง Grade เลย)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — selectedChoice := verdictChoice ตรวจผ่าน choiceOf ; Cover ที่แก้เป็น 0 ทุกหมวดได้ Grade ต่างจาก Cover เดิมที่เป็น 2 ; แถวเลื่อนสถานะพา verdictChoice และ description ไปด้วย (run 007)
+ผลที่บันทึกไว้: 23/23, run 006, 24 ส.ค. 2569 · ชุดนี้ตอนนี้ 30/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>003-FR-5
-ระดับที่ 1 ไม่สรุปผล ODPC สรุปผลและแก้ทับ</t>
+ระดับที่ 1 ไม่สรุปผล ODPC สรุปผลและแก้ทับ  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -1128,56 +1314,58 @@
           <t>ระดับที่ 1 แก้ได้แค่ของตัวเองและเฉพาะตอน Cover ยัง in_review ส่วน ODPC แก้ทับได้ทุกข้อ ที่ยังไม่เป็น finished และเป็นคนเดียวที่เปลี่ยนสถานะ Cover ได้ คำตอบที่ finished แล้วใครก็แก้ไม่ได้</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — กรณีแก้ไขไม่ได้ 400 และ ODPC แก้ทับ 200 ; verdict — ระดับที่ 1 ได้ 403 การเลื่อนสถานะ และการปิดช่องว่าง (แก้ไขโดย 008-FR-2)
-ผลที่บันทึกไว้: 16/16, bolt 023, 7 ก.ค. 2569</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — กรณีแก้ไขไม่ได้ 400 และ ODPC แก้ทับ 200 ; verdict — ระดับที่ 1 ได้ 403 การเลื่อนสถานะ และการปิดช่องว่าง (⟲ ADR-0012 ทำให้การแก้คะแนนอยู่ใต้เงื่อนไขของ recommended ด้วย คือเจ้าของหรือ ODPC เท่านั้น เข้มขึ้นกว่าเดิมที่ใครดูแลหมวดนั้นก็แก้ได้)
+ผลที่บันทึกไว้: 26/26 + 30/30, run 005 / 009</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="94" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>003-FR-6
-วงจรต่อรอง</t>
+วงจรต่อรอง  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>โรงงานเลือกยอมรับคะแนนที่เสนอ (ได้ recommended และต้องผ่านการตรวจไฟล์ตามระดับคะแนนใหม่) หรือโต้แย้งเพื่อตอบใหม่ (กลับไป in_review) วนได้ไม่จำกัดรอบ จบได้ด้วยการตกลงกันเท่านั้น</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>ตรวจด้วยการอ่านโค้ด
-หลักฐาน: อ่านโค้ดใน bolt 009 จำนวน 5 เกณฑ์ + 1 กรณีขอบเขต
-ผลที่บันทึกไว้: ยังไม่มีกรณีทดสอบที่รันได้ — ดู G-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="58" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+          <t>เดิม: การแก้คะแนนเปิดวงจรต่อรองที่โรงงานเลือกยอมรับหรือโต้แย้งได้ วนไม่จำกัดรอบ
+⟲ ADR-0012 เลิกใช้วงจรนี้กับการแก้คะแนน คำวินิจฉัยของผู้ตรวจถือเป็นที่สุด โรงงานไม่มีอะไรให้ต่อรองและไม่เสียไฟล์ ส่วนวงจรต่อรองยังอยู่ครบสำหรับ hard reject ซึ่งโรงงานต้องทำใหม่พร้อมหลักฐานใหม่</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: answer.integration — describe “negotiate — a settled score change admits no factory response” 4 กรณี ครอบคลุมทั้ง accept และ redo ทั้งรูปแบบใหม่ (recommended) และรูปแบบเดิม (rejected + verdictChoice) ส่วน hard reject ยังใช้ข้อความเดิม หมายเหตุ: ก่อน run 007 เส้นทาง negotiate ไม่เคยมีเทสต์เลยสักกรณี
+ผลที่บันทึกไว้: 9/9, run 007, 24 ส.ค. 2569 — ปิดช่องว่าง G-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>003-FR-7
-การจัดการไฟล์ตอนส่งกลับ</t>
+การจัดการไฟล์ตอนส่งกลับ  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>change-score เก็บไฟล์ไว้ ส่วน reject ลบไฟล์ออกจาก MinIO ตอน ODPC สรุปผล และงานไฟล์ทั้งหมดต้องอยู่นอกทรานแซกชัน ส่วนตอนโรงงานตอบใหม่ก็จัดการไฟล์ได้อิสระ</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — กรณีลบไฟล์ และกรณียกเลิกเมื่อ MinIO ล้มเหลว (ขาที่โรงงานจัดการไฟล์ตอนตอบใหม่ยังใช้การอ่านโค้ด ; แก้ไขโดย 010-FR-1)
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
+          <t>งานไฟล์ทั้งหมดอยู่นอกทรานแซกชัน
+⟲ ADR-0012 คืนกติกาเดิมของ ADR-0005 — change-score เก็บไฟล์ไว้ ส่วน hard reject ลบไฟล์ตอนสรุปผล และตั้งแต่ run 009 ยังลบใบรับรองมาตรฐาน ที่คำถามข้อนั้นอ้างถึงและโรงงานแจ้งไว้ด้วย</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — ชุดที่ลบคือ hard reject เท่านั้น แถว rejected ที่มี verdictChoice ยังเก็บไฟล์ไว้ ; กรณี MinIO ล้มเหลวยังยกเลิกก่อนแตะฐานข้อมูล ; run 009 เพิ่มการลบใบรับรองมาตรฐาน 7 กรณี
+ผลที่บันทึกไว้: 23/23 run 006 → 30/30 run 009, 25 ส.ค. 2569</t>
         </is>
       </c>
     </row>
     <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>003-FR-8
 เงื่อนไขการส่งซ้ำ</t>
@@ -1188,16 +1376,16 @@
           <t>โรงงานส่งซ้ำได้เมื่อไม่เหลือคำตอบสถานะ rejected แล้ว พอส่งแล้ว Cover กลับไป in_review ส่วนคำตอบที่ finished แล้วจะติดตัวไปเลยไม่ต้องตรวจซ้ำ</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>ตรวจด้วยการอ่านโค้ด
 หลักฐาน: อ่านโค้ดใน bolt 009 จำนวน 4 เกณฑ์ + 1 กรณีขอบเขต
-ผลที่บันทึกไว้: ยังไม่มีกรณีทดสอบที่รันได้ — ดู G-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+ผลที่บันทึกไว้: ยังไม่มีกรณีทดสอบที่รันได้ — ดู G-2 (เป็นข้อสุดท้ายที่เหลือในช่องว่างนี้)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="80" customHeight="1">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>003-FR-9
 ระดับรางวัลตอนสรุปผล</t>
@@ -1208,31 +1396,32 @@
           <t>gold ต้องทุกหมวด &gt; 80% รวม ≥ 90% และได้เต็มทุกข้อที่เป็น special · silver ทุกหมวด &gt; 60% รวม ≥ 80% · certificate รวม ≥ 60% · joined รวม &lt; 60% ไล่จากบนลงล่างอย่างเคร่งครัด และถ้า Cover กลับไป in_progress จะไม่มี Grade</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>ยืนยันบางส่วน
-หลักฐาน: score.test.ts — เกณฑ์และค่าขอบ ; verdict — การสรุปผลคืนค่า Grade แต่ตรวจแค่ว่าค่าอยู่ในชุดที่ถูกต้อง ยังไม่เทียบกับค่าที่ควรได้ (G-3)
-ผลที่บันทึกไว้: 24/24 แบบแยกอิสระ, 15 ก.ค. 2569</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="58" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+หลักฐาน: score.test.ts — เกณฑ์และค่าขอบ 27 กรณี ; verdict — การสรุปผลคืนค่า Grade และ run 006 พิสูจน์เพิ่มว่า Grade เปลี่ยนตามคะแนนที่ผู้ตรวจแก้ แต่ยังไม่มีกรณีที่เทียบข้อมูลตั้งต้นกับค่า Grade ที่ควรได้แบบเจาะจง (G-3)
+ผลที่บันทึกไว้: 27/27 แบบแยกอิสระ · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="80" customHeight="1">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>003-FR-10
-อีเมลทุกครั้งที่ ODPC สรุปผล</t>
+อีเมลทุกครั้งที่ ODPC สรุปผล  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>finished ส่งแบบ “ผ่านพร้อมระดับรางวัล” ส่วน in_progress ส่งแบบ “ต้องแก้ไข” และต้องไม่ส่งเมื่อระดับที่ 1 บันทึกหรือโรงงานส่งซ้ำ ส่งผ่านคิว BullMQ เดิม</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — verdict-result-finished และ verdict-result-in-progress อย่างละหนึ่งฉบับ พร้อมตรวจเนื้อหา ; save — ไม่มีอีเมลตอนบันทึก
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
+          <t>finished ส่งแบบ “ผ่านพร้อมระดับรางวัล” ส่วน in_progress ส่งแบบ “ต้องแก้ไข” และต้องไม่ส่งเมื่อระดับที่ 1 บันทึกหรือโรงงานส่งซ้ำ
+⟲ เดิมตั้งใจให้อีเมล finished ไล่รายการข้อที่ถูกแก้คะแนนด้วย แต่ human ตัดสินใจ 24 ส.ค. 2569 ว่าไม่ต้องแก้อีเมล ใช้การอ่านข้อมูลกลับแทน</t>
+        </is>
+      </c>
+      <c r="C14" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — verdict-result-finished และ verdict-result-in-progress อย่างละหนึ่งฉบับ ; save — ไม่มีอีเมลตอนบันทึก ; run 008 ยืนยันว่า payload อีเมลไม่เปลี่ยนเลย และโรงงานอ่านค่าที่แก้แล้วกลับมาได้จริง
+ผลที่บันทึกไว้: 30/30 + 9/9, run 008, 24 ส.ค. 2569</t>
         </is>
       </c>
     </row>
@@ -1252,8 +1441,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1263,32 +1452,32 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>เปิดช่องทางที่สองเข้าสู่กระบวนการเดิม โดยไม่เพิ่มกติกาการตรวจใหม่เลยสักข้อ ใช้โค้ดร่วมกับ ODPC จริง จุดที่ยังอ่อนจึงไปกองที่ขอบ คือสิทธิ์เข้าใช้กับการบันทึกว่าใครเป็นคนทำ</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>004-FR-1
 บริบทผู้ตรวจสังเคราะห์</t>
@@ -1299,7 +1488,7 @@
           <t>เวลาผู้ดูแลเข้ามา ให้ประกอบบริบทเป็น {accountId, level: "ODPC", region: null} แทนการไปหาในตาราง evaluators เพื่อไม่ให้โดนปฏิเสธด้วย 404 "invalid evaluator" และต้องได้สิทธิ์ครบ 5 หมวดแบบ ODPC ส่วนเส้นทางเดิมของผู้ประเมินต้องไม่เปลี่ยน</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: evaluator-review.integration — กรณี adminReviewerContext
@@ -1308,7 +1497,7 @@
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>004-FR-2
 เข้าถึงข้ามเขตระดับประเทศ</t>
@@ -1319,7 +1508,7 @@
           <t>พอ region เป็น null ให้ข้ามการเช็กเขต เหลือแค่เช็กว่า Cover มีอยู่จริง ถ้าไม่มีก็ยังคืน 404 เหมือนเดิม ส่วนผู้ประเมินตัวจริงยังถูกจำกัดเขตไม่เปลี่ยน</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: evaluator-review.integration — region null + ไม่มี cover → 404 และผู้ประเมินผิดเขต → 404
@@ -1327,8 +1516,8 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="64" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>004-FR-3
 เส้นทางรายการคำตอบฝั่งผู้ดูแล</t>
@@ -1339,16 +1528,16 @@
           <t>GET …/admins/covers/:id/answers อยู่ใต้ adminGuard (Role.DOED) ใช้ AnswerViewSchema ตัวเดิม และคืนคำตอบครบทั้ง 5 หมวดเพราะ ODPC ดูแลทุกหมวด</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>ยืนยันบางส่วน
 หลักฐาน: evaluator-review.integration — การอ่านฝั่งผู้ดูแล + Value.Check(AnswerViewSchema) ; standards — ความเท่าเทียมของฝั่งผู้ดูแล  ตัว adminGuard เองยังไม่มีการตรวจ (D-01 / G-7)
-ผลที่บันทึกไว้: 50/50, bolt 022</t>
+ผลที่บันทึกไว้: 10/10 + 6/6 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>004-FR-4
 เส้นทางบันทึกผลแบบชุดฝั่งผู้ดูแล</t>
@@ -1359,7 +1548,7 @@
           <t>รับ body แบบเดียวกับฝั่งผู้ประเมิน แล้วขับเคลื่อนการสรุปผลแบบ ODPC เต็มรูปแบบ ทั้งการแก้ทับ การปิดช่องว่าง การลบไฟล์ การเปลี่ยนสถานะ Grade และอีเมล</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>เลิกใช้แล้ว
 หลักฐาน: bolt 012 ตรวจไว้ (6/6) ต่อมาเส้นทางแบบชุดถูกลบใน bolt 021 และชุดทดสอบนั้นก็ถูกแทนที่ไปด้วย
@@ -1368,7 +1557,7 @@
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>004-FR-5
 เท่าเทียมกับ ODPC พอดี ไม่มีอำนาจเกิน</t>
@@ -1379,16 +1568,16 @@
           <t>คำตอบที่ finished แล้วผู้ดูแลก็แก้ไม่ได้เหมือนกัน ไม่มีโหมดร่างแยก และไม่มีทางลัดพิเศษแม้ในเขตที่ไม่มี ODPC</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: save — แก้ไขไม่ได้ 400 สำหรับทุกระดับ ; verdict — การสรุปผลฝั่งผู้ดูแลผ่านเงื่อนไขชุดเดียวกัน
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="78" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+ผลที่บันทึกไว้: 26/26 + 30/30 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>004-FR-6
 บันทึกว่าใครเป็นคนทำ</t>
@@ -1399,10 +1588,10 @@
           <t>เขียน accountId ของผู้ดูแลลง answerLogs.eval_id และ coverLogs.evaluatorId โดยใช้คอลัมน์เดิมที่เป็น int ธรรมดาไม่มี FK จึงไม่ต้องแก้ฐานข้อมูล และไม่ใส่ตัวบอกว่าเป็นผู้ดูแลหรือ ODPC</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>ยืนยันบางส่วน
-หลักฐาน: verdict — ล็อกการเลื่อนสถานะบันทึกผู้สรุปผล (eval_id) ส่วนการตรวจ coverLogs.evaluatorId เฉพาะฝั่งผู้ดูแลหายไปตอน bolt 021 แทนที่ชุดทดสอบของ bolt 012 → นี่คือ G-1 จุดที่ควรแก้ก่อนใคร
+หลักฐาน: verdict — ล็อกการเลื่อนสถานะบันทึกผู้สรุปผล (eval_id) ส่วนการตรวจ coverLogs.evaluatorId เฉพาะฝั่งผู้ดูแลหายไปตอน bolt 021 แทนที่ชุดทดสอบของ bolt 012 → นี่คือ G-1 ยังเปิดอยู่ และงานของ intent ล่าสุดก็ไม่ได้แตะจุดนี้
 ผลที่บันทึกไว้: bolt 012 6/6 (19 มิ.ย. 2569) แล้วถูกแทนที่</t>
         </is>
       </c>
@@ -1423,8 +1612,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1434,32 +1623,32 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>เปลี่ยนวิธีเขียนข้อมูลทั้งหมด จากเดิมที่ต้องกดส่งทีเดียวทั้งชุด มาเป็นบันทึกทีละข้อที่เก็บผลทันที แล้วแยกขั้นสรุปผลออกมาต่างหาก ครบ 9 จาก 9 เป็นแกนที่แข็งแรงที่สุดของโมดูล</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>008-FR-1
 บันทึกทีละข้อ</t>
@@ -1470,56 +1659,58 @@
           <t>POST …/answers/:answerId/verdict รับคำวินิจฉัยข้อเดียว เขียน answerLogs หนึ่งแถวแล้วคืนสถานะใหม่ ถ้าเสนอคะแนนเท่าเดิมให้ตอบ 400 เพราะควรใช้ approve แทน และห้ามมีผลข้างเคียงอื่นเลย ไม่แตะไฟล์ ไม่เปลี่ยนสถานะ Cover ไม่ส่งอีเมล</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — กรณีคำวินิจฉัย, no-op 400, นอกขอบเขต 403, ไม่อยู่ใน cover 400, ผิดเขต 404 และกรณีไม่มีผลข้างเคียง
-ผลที่บันทึกไว้: 19/19, bolt 019, 2 ก.ค. 2569</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — กรณีคำวินิจฉัย, no-op 400, นอกขอบเขต 403, ไม่อยู่ใน cover 400, ผิดเขต 404 และกรณีไม่มีผลข้างเคียง (coverLogs ไม่เพิ่มขึ้นเลย)
+ผลที่บันทึกไว้: 26/26, run 005, 24 ส.ค. 2569</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>008-FR-2
-บันทึกแล้วได้สถานะทันที ไม่มีสถานะร่าง</t>
+บันทึกแล้วได้สถานะทันที ไม่มีสถานะร่าง  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>approve ได้ recommended สำหรับทุกคนรวมถึง ODPC ด้วย · change-score ได้ rejected พร้อมคะแนนเสนอและคำอธิบาย เก็บไฟล์ไว้ · reject ได้ rejected แบบไม่มีคะแนนเสนอ และยังไม่ลบไฟล์ตอนนี้</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — ระดับที่ 1 approve → recommended และ ODPC approve → recommended
-ผลที่บันทึกไว้: 19/19, bolt 019</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+          <t>approve ได้ recommended สำหรับทุกคนรวมถึง ODPC ด้วย
+⟲ ADR-0012 ย้าย change-score มาอยู่ฝั่งเดียวกัน คือได้ recommended พร้อมเก็บไฟล์ไว้ เหลือแค่ reject ที่ได้ rejected และยังไม่ลบไฟล์ตอนบันทึก</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — ระดับที่ 1 approve → recommended, ODPC approve → recommended และ change_score → recommended
+ผลที่บันทึกไว้: 26/26, run 005</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>008-FR-3
-ตรวจสิทธิ์แก้ไขจากคนที่บันทึกไว้ก่อน</t>
+ตรวจสิทธิ์แก้ไขจากคนที่บันทึกไว้ก่อน  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>finished ห้ามทุกคน · recommended แก้ได้เฉพาะคนที่บันทึกไว้เองหรือ ODPC (กันระดับที่ 1 ไปรื้อของที่โรงงานยอมรับไปแล้ว) · rejected กับ in_review ใครที่ดูแลหมวดนั้นก็แก้ได้</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — 5 กรณีครอบคลุมทั้ง 4 สาขาเงื่อนไข
-ผลที่บันทึกไว้: 19/19, bolt 019</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+          <t>finished ห้ามทุกคน · recommended แก้ได้เฉพาะคนที่บันทึกไว้เองหรือ ODPC (กันระดับที่ 1 ไปรื้อของที่โรงงานยอมรับไปแล้ว) · rejected กับ in_review ใครที่ดูแลหมวดนั้นก็แก้ได้
+⟲ พอ change-score ย้ายไปเป็น recommended มันก็เข้ามาอยู่ใต้กติกานี้ด้วย เข้มขึ้นกว่าเดิม</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — 5 กรณีเดิมครอบคลุมทั้ง 4 สาขาเงื่อนไข บวกกรณีใหม่ที่ระดับที่ 1 คนอื่นแก้ score change ของคนอื่นไม่ได้ (403) แต่เจ้าของแก้ได้ (200)
+ผลที่บันทึกไว้: 26/26, run 005</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>008-FR-4
 การสรุปผลทั้ง Cover</t>
@@ -1530,16 +1721,16 @@
           <t>POST …/finalize body ว่าง เฉพาะ ODPC กับผู้ดูแล อ่านจากล็อกที่บันทึกไว้แล้ว ถ้ายังมีข้อไหน in_review ให้ตอบ 400 ไม่แต่งคำวินิจฉัยขึ้นมาเอง จากนั้นเลื่อน recommended เป็น finished ลบไฟล์ของข้อที่ถูกปฏิเสธ เขียนสถานะ Cover คำนวณ Grade และส่งอีเมล</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — 16 กรณีครอบคลุมสิทธิ์ เงื่อนไขปิดกั้น การเลื่อนสถานะ ผลลัพธ์ทั้งสองแบบ การลบไฟล์ และความเป็นอะตอมมิก
-ผลที่บันทึกไว้: 16/16, bolt 023, 7 ก.ค. 2569</t>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — 30 กรณีครอบคลุมสิทธิ์ เงื่อนไขปิดกั้น การเลื่อนสถานะ ผลลัพธ์ทั้งสองแบบ การลบไฟล์ ความเป็นอะตอมมิก และการสรุปผลซ้ำ (run 006 เจอและแก้บั๊กล็อกซ้ำที่ตัวเองทำขึ้น)
+ผลที่บันทึกไว้: 30/30, run 009, 25 ส.ค. 2569 (ชุดนี้โต 17 → 23 → 30)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="18" t="inlineStr">
         <is>
           <t>008-FR-5
 finished เขียนได้จากการสรุปผลเท่านั้น</t>
@@ -1550,36 +1741,37 @@
           <t>ไม่มีเส้นทางบันทึกไหนเขียน finished ได้ และ ODPC ที่กด approve ไว้ ก็ยังกลับมาแก้ได้จนกว่าจะสรุปผล ส่วนการเปลี่ยนสถานะ Cover ก็เขียนได้จากการสรุปผลอย่างเดียว</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: save — ODPC approve ไม่เคยได้ finished ; verdict — กรณีคู่ของ FR-5 (ตรวจสองทาง)
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="58" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+ผลที่บันทึกไว้: 26/26 + 30/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>008-FR-6
-เลื่อนการลบไฟล์ไปตอนสรุปผล</t>
+เลื่อนการลบไฟล์ไปตอนสรุปผล  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ตอนบันทึกไม่แตะ MinIO เลย ถ้าข้อที่เคยถูกปฏิเสธถูกแก้ทับก่อนสรุปผล ไฟล์ต้องยังอยู่ เพราะชุดที่จะลบคำนวณจากสถานะสุดท้ายเท่านั้น</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: save — ไม่มีผลข้างเคียง ; verdict — คำนวณชุดที่ลบจากสถานะสุดท้าย และกรณีแก้ทับก่อนสรุปผลยังเก็บไฟล์ไว้ (แก้ไขโดย 010-FR-1)
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="64" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+          <t>ตอนบันทึกไม่แตะ MinIO เลย และชุดที่จะลบคำนวณจากสถานะสุดท้ายเท่านั้น
+⟲ ADR-0012 บีบชุดที่ลบให้เหลือแค่ hard reject โดยจำแนกด้วย status = rejected AND verdict_choice IS NULL ซึ่งจงใจเขียนแบบนี้เพื่อให้แถวเก่า ที่บันทึกไว้ก่อนเปลี่ยนกติกา ยังถูกจัดเป็นการแก้คะแนนและไม่เสียไฟล์ โดยไม่ต้อง backfill</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — แถว rejected ที่มี verdictChoice ยังเก็บไฟล์ไว้ มีแต่ reject ที่ verdict เป็น null ที่ถูกลบ ; มีกรณีเฉพาะสำหรับแถวรูปแบบเก่าว่าจบงานได้โดยไม่ต้อง backfill
+ผลที่บันทึกไว้: 23/23, run 006, 24 ส.ค. 2569</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="18" t="inlineStr">
         <is>
           <t>008-FR-7
 ใช้ได้ทั้งสองฝั่ง</t>
@@ -1590,16 +1782,16 @@
           <t>ฝั่งผู้ประเมินหาบริบทผ่าน resolveEvaluator ฝั่งผู้ดูแลผ่าน adminReviewerContext แต่เรียก service ตัวเดียวกัน พฤติกรรมการบันทึกเหมือนกันเป๊ะ และการสรุปผลสงวนไว้ให้ ODPC กับผู้ดูแลทั้งสองฝั่ง</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: verdict — กรณีสรุปผลฝั่งผู้ดูแล ; การยิงคำขอใน bolt 021 ยืนยันว่าเส้นทางทั้งสองฝั่งลงทะเบียนแล้ว (ระดับ service ; ตัว guard ยังไม่มีการตรวจ — G-7)
-ผลที่บันทึกไว้: 44/44, bolt 021, 2 ก.ค. 2569</t>
+ผลที่บันทึกไว้: 30/30 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="12" ht="58" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>008-FR-8
 ถอดเส้นทางแบบชุดออก</t>
@@ -1610,7 +1802,7 @@
           <t>ลบ POST …/covers/:id/verdict ทั้งสองฝั่ง พร้อม VerdictBatchSchema และกรณี 400 เรื่อง answerId ซ้ำ แล้วเพิ่ม FinalizeSchema เข้ามาแทน</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: การยิงคำขอ bolt 021 — เส้นทางแบบชุดทั้งสองได้ 404 ไม่มีไฟล์ทดสอบไหนอ้างถึง VerdictBatchSchema และ API.md ก็ไม่เหลือการอ้างอิง
@@ -1619,7 +1811,7 @@
       </c>
     </row>
     <row r="13" ht="58" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="18" t="inlineStr">
         <is>
           <t>008-FR-9
 รายการคำตอบไม่เปลี่ยน</t>
@@ -1630,11 +1822,11 @@
           <t>ยังคืนสถานะปัจจุบันของแต่ละข้อเหมือนเดิม เพื่อให้ผู้ประเมินกลับมาตรวจต่อจากจุดเดิมได้ ไม่เปลี่ยนการกรอง การเลือกฟิลด์ หรือขอบเขตเขต/หมวด</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: evaluator-review.integration — การทดสอบถดถอยของ getAnswers (การกรอง การเลือกฟิลด์ และขอบเขต)
-ผลที่บันทึกไว้: 50/50, bolt 022</t>
+ผลที่บันทึกไว้: 10/10 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
@@ -1654,8 +1846,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1665,32 +1857,32 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>แก้ปัญหาที่ผู้ตรวจต้องสลับหน้าจอไปดูใบรับรองมาตรฐานของโรงงาน เป็นงานอ่านอย่างเดียว ไม่แตะฐานข้อมูล ปิดจบได้ครบที่สุดในบรรดา intent ทั้งหมด</t>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>แก้ปัญหาที่ผู้ตรวจต้องสลับหน้าจอไปดูใบรับรองมาตรฐานของโรงงาน เป็นงานอ่านอย่างเดียว ไม่แตะฐานข้อมูล ต่อมา run 009 ต่อยอดข้อมูลชุดนี้ไปใช้ตอนลบไฟล์เมื่อ hard reject</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="18" t="inlineStr">
         <is>
           <t>009-FR-1
 แสดงไฟล์มาตรฐานของโรงงาน</t>
@@ -1701,16 +1893,16 @@
           <t>คืนเป็น { standard, fileName } โดย standard ใช้ค่า enum ตรง ๆ ไม่ใช่ชื่อไทย และแสดงเฉพาะมาตรฐานที่โรงงานทั้งแจ้งไว้และอัปโหลดไฟล์แล้ว ส่วนการเปิดดูไฟล์ยังใช้ /file/presigned-url ตัวเดิม</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: standards — ตัดกรณีแจ้งแต่ไม่มีไฟล์ ตัดกรณีมีไฟล์แต่ไม่ได้แจ้ง และแสดงกรณีที่ครบทั้งสองเงื่อนไข
-ผลที่บันทึกไว้: 50/50, bolt 022, 3 ก.ค. 2569</t>
+ผลที่บันทึกไว้: 6/6 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>009-FR-2
 เปลี่ยนรูปแบบผลลัพธ์เป็น { answers, standards }</t>
@@ -1721,16 +1913,16 @@
           <t>จากเดิมที่คืน array เปล่า ๆ มาเป็น object ที่ห่อสองก้อนไว้ โดยส่วน answers ต้องเหมือนเดิมทุกอย่าง ทั้งลำดับ การกรอง และฟิลด์ ถือเป็น breaking change ต้อง regen เอกสาร API ด้วย</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: standards — กรณีตรวจรูปแบบ ; evaluator-review.integration — การทดสอบถดถอยที่ปรับแล้ว
-ผลที่บันทึกไว้: 50/50, bolt 022</t>
+ผลที่บันทึกไว้: 6/6 + 10/10</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>009-FR-3
 ใช้ได้ทั้งสองฝั่งและเหมือนกัน</t>
@@ -1741,16 +1933,16 @@
           <t>มาตรฐานเป็นข้อมูลระดับโรงงาน ผู้ประเมินระดับที่ 1 ที่เห็นคำตอบแค่หมวดตัวเอง ก็ยังต้องเห็นมาตรฐานครบทุกใบ และกติกาการเข้าถึง Cover ยังเหมือนเดิม ไม่มีข้อมูลรั่ว</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>ยืนยันแล้ว
 หลักฐาน: standards — ระดับที่ 1 เห็นมาตรฐานครบ ผู้ดูแลได้ผลเท่ากับ ODPC ระดับเขต และผิดเขต 404 โดยไม่รั่วข้อมูล
-ผลที่บันทึกไว้: 50/50, bolt 022</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="64" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+ผลที่บันทึกไว้: 6/6 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>009-FR-4
 อ่านอย่างเดียวจากข้อมูลการลงทะเบียน</t>
@@ -1758,14 +1950,15 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ดึงจากคอลัมน์ standard* กับ fileStandard*Url ที่มีอยู่แล้ว ไม่เพิ่มตาราง ไม่เพิ่ม endpoint อัปโหลด join covers → enrolls ในเส้นทางเดิม และต้องไม่เกิด N+1</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
+          <t>ดึงจากคอลัมน์ standard* กับ fileStandard*Url ที่มีอยู่แล้ว ไม่เพิ่มตาราง ไม่เพิ่ม endpoint อัปโหลด join covers → enrolls ในเส้นทางเดิม และต้องไม่เกิด N+1
+หมายเหตุ: run 009 พบว่าการ spread STANDARD_ENROLL_COLUMNS เข้าไปใน select ทำให้ Drizzle เดาชนิดข้อมูลไม่ออก จึงต้องเขียนทั้ง 11 คู่ออกมาตรง ๆ</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>ยืนยันบางส่วน
-หลักฐาน: standards — cover ที่ไม่มีคำตอบก็ยังคืนมาตรฐาน ส่วนเรื่องไม่เกิด N+1 เป็นคุณสมบัติเชิงโครงสร้างของ STANDARD_ENROLL_COLUMNS ที่ยืนยันด้วยการอ่านโค้ด (G-4)
-ผลที่บันทึกไว้: 50/50, bolt 022</t>
+หลักฐาน: standards — cover ที่ไม่มีคำตอบก็ยังคืนมาตรฐาน ส่วนเรื่องไม่เกิด N+1 เป็นคุณสมบัติเชิงโครงสร้างที่ยืนยันด้วยการอ่านโค้ด (G-4)
+ผลที่บันทึกไว้: 6/6 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
@@ -1785,83 +1978,85 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Intent 010 — ลบไฟล์หลักฐานเมื่อปรับคะแนน</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>intent ที่เล็กที่สุด แก้เงื่อนไขเดียวในโค้ด เกิดจากการกลับคำตัดสินใจเดิมใน ADR-0005 ที่เคยให้ change-score เก็บไฟล์ไว้ (บันทึกไว้เป็น ADR-0006)</t>
+          <t>Intent 010 — ลบไฟล์หลักฐานเมื่อปรับคะแนน  ⟲ ถูกกลับคำทั้ง intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>⚠️ intent นี้ถูก ADR-0012 ยกเลิก — ADR-0006 ที่เป็นฐานของมันถูกแทนที่ทั้งฉบับเมื่อ 25 ส.ค. 2569 สาเหตุคือมันไปทำให้วงจรต่อรองของ ADR-0004 พังโดยไม่มีใครสังเกต และทำให้โรงงานเสียหลักฐาน ทุกครั้งที่ผู้ตรวจแก้คะแนน เป็นแบบนี้อยู่ราว 6 สัปดาห์บน production</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>010-FR-1
-ขยายเงื่อนไขการลบ</t>
+ขยายเงื่อนไขการลบ  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>เปลี่ยนจาก “ปฏิเสธและไม่มีคะแนนเสนอ” มาเป็น “ปฏิเสธทุกกรณี” ดังนั้น change-score ก็โดนลบไฟล์และล้างคอลัมน์ fileUrl* ด้วย ส่วนข้อที่เป็น recommended หรือ finished ยังไม่แตะ ถ้าถูกแก้กลับเป็น approve ก่อนสรุปผลก็ยังเก็บไฟล์ไว้ และยังลบนอกทรานแซกชันเหมือนเดิม</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — ทั้ง change-score และการปฏิเสธโดยตรงถูกลบ ส่วน recommended ยังอยู่ และกรณีแก้ทับก่อนสรุปผลยังเก็บไฟล์ไว้
-ผลที่บันทึกไว้: 16/16, bolt 023, 7 ก.ค. 2569</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+          <t>เดิม: เปลี่ยนจาก “ปฏิเสธและไม่มีคะแนนเสนอ” มาเป็น “ปฏิเสธทุกกรณี” ทำให้ change-score โดนลบไฟล์และล้างคอลัมน์ fileUrl* ด้วย
+⟲ กลับคำทั้งข้อ ตอนนี้ change-score เก็บไฟล์ไว้อีกครั้ง เงื่อนไขการลบกลับไปเป็น status = rejected AND verdict_choice IS NULL ตาม 008-FR-6</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>เลิกใช้แล้ว
+หลักฐาน: เคยยืนยันไว้ที่ 16/16 bolt 023 (7 ก.ค. 2569) ต่อมา run 006 เขียนกรณีทดสอบข้อนี้ใหม่ให้ตรวจตรงกันข้าม คือไฟล์ต้องยังอยู่
+ผลที่บันทึกไว้: ยกเลิกแล้ว — แทนด้วย ADR-0012 / 008-FR-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>010-FR-2
-สถานะ Cover และ Grade ยังเหมือนเดิม</t>
+สถานะ Cover และ Grade ยังเหมือนเดิม  ⟲ ปรับตาม ADR-0012</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>intent นี้แตะแค่เรื่องไฟล์ Cover ที่มี change-score ยังต้องกลับไป in_progress ได้ Grade เป็น null และส่งอีเมลแบบต้องแก้ไข เหมือนเดิมทุกอย่าง</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — มีข้อถูกปฏิเสธ ≥ 1 → in_progress + Grade เป็น null ; ทุกข้อ recommended → finished + Grade (ผ่านโดยไม่ต้องแก้โค้ด)
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
+          <t>เดิม: Cover ที่มี change-score ยังต้องกลับไป in_progress ได้ Grade เป็น null และส่งอีเมลแบบต้องแก้ไข
+⟲ กลับคำ ตอนนี้ Cover ที่มีแต่ approve กับ change-score ไปถึง finished ได้ในรอบเดียว พร้อม Grade ที่คิดจากคะแนนที่ผู้ตรวจแก้</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>เลิกใช้แล้ว
+หลักฐาน: verdict — Cover ที่มีแต่ score change จบเป็น finished ในรอบเดียว ไม่มีการเด้งกลับ (run 006)
+ผลที่บันทึกไว้: ยกเลิกแล้ว — แทนด้วย SCF-2</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>010-FR-3
 ทั้งสองฝั่งยังเท่าเทียมกัน</t>
@@ -1869,14 +2064,14 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>เพราะ finalize เป็นโค้ดตัวเดียวกัน จึงต้องไม่มีการแยกตรรกะรายฝั่งเพิ่มเข้ามา</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
-        <is>
-          <t>ยืนยันแล้ว
-หลักฐาน: verdict — กรณีสรุปผลฝั่งผู้ดูแล ไม่ได้แก้อะไรและยังผ่านอยู่
-ผลที่บันทึกไว้: 16/16, bolt 023</t>
+          <t>เพราะ finalize เป็นโค้ดตัวเดียวกัน จึงต้องไม่มีการแยกตรรกะรายฝั่งเพิ่มเข้ามา ข้อนี้ยังใช้อยู่ เพราะเป็นกติกาเชิงโครงสร้างที่ไม่ขึ้นกับเงื่อนไขการลบไฟล์</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — กรณีสรุปผลฝั่งผู้ดูแล ยังผ่านอยู่หลังการเปลี่ยนแปลงของ ADR-0012
+ผลที่บันทึกไว้: 30/30, run 009, 25 ส.ค. 2569</t>
         </is>
       </c>
     </row>
@@ -1896,8 +2091,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1907,35 +2102,35 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>intent ป้องกันปัญหา ไม่ใช่แก้บั๊กที่เกิดแล้ว โค้ดปัจจุบันทำถูกอยู่แล้วในเส้นทางหลัก แต่ยังไม่เคยถูกเขียนเป็นสัญญาที่ชัดเจนและทดสอบครบทุกช่องทาง ทั้ง 5 ข้อยังไม่ได้รัน</t>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>intent ป้องกันปัญหา ไม่ใช่แก้บั๊กที่เกิดแล้ว รอบก่อนยังอยู่ในสถานะยังไม่ได้รัน ตอนนี้งานถูก commit เข้า main แล้วและอยู่ในชุดทดสอบเต็มที่ผ่าน 537/0 จึงเลื่อนเป็นยืนยันแล้วทั้งหมด</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>requirement</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>ผลการทดสอบ</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="5" ht="66" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>011-FR-1
-CoverLog ล่าสุดเป็นตัวตัดสินสิทธิ์ Grade</t>
+CoverLog ล่าสุดเป็นตัวตัดสินสิทธิ์ Grade  ✓ รันแล้ว</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
@@ -1943,19 +2138,19 @@
           <t>ดูจากแถวที่ id สูงสุด ไม่ใช้เวลาประทับ ดังนั้นล็อก finished เก่าที่มีล็อกใหม่กว่ามาทับ จะไม่ทำให้ Cover ได้ Grade ส่วน Cover ที่ยังไม่มีล็อกเลยก็ใช้ค่าตั้งต้น in_progress เหมือนเดิม</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>ยังไม่ได้รัน
-หลักฐาน: score.integration — กรณี intent-011 จงใจสลับเวลาประทับ เพื่อพิสูจน์ว่าใช้ลำดับ id จริง
-ผลที่บันทึกไว้: ยังไม่ commit และยังไม่มีบันทึกผลการรัน</t>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: score.integration — describe “Intent 011 — latest CoverLog gates Grade across every score surface” จงใจสลับเวลาประทับเพื่อพิสูจน์ว่าใช้ลำดับ id จริง
+ผลที่บันทึกไว้: 16/16 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>011-FR-2
-รายงานคะแนนคืน Grade เฉพาะ Cover ที่ finished</t>
+รายงานคะแนนคืน Grade เฉพาะ Cover ที่ finished  ✓ รันแล้ว</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
@@ -1963,19 +2158,19 @@
           <t>in_review ยังได้คะแนนตัวเลขตามปกติแต่ grade เป็น null · finished ได้ทั้งคะแนนและ Grade · in_progress ยังตอบ 400 เหมือนเดิม และรายการของผู้ประเมิน เจ้าหน้าที่จังหวัด และผู้ดูแล ก็ใช้กติกาเดียวกัน</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>ยังไม่ได้รัน
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
 หลักฐาน: score.integration — กรณีเดียวกันไล่ตรวจโรงงาน เขต จังหวัด และผู้ดูแล ผ่านสถานะ finished → in_review → in_progress
-ผลที่บันทึกไว้: ยังไม่ commit</t>
+ผลที่บันทึกไว้: 16/16 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>011-FR-3
-การสรุปผลคืนและส่ง Grade เฉพาะเมื่อ commit finished แล้ว</t>
+การสรุปผลคืนและส่ง Grade เฉพาะเมื่อ commit finished แล้ว  ✓ รันแล้ว</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -1983,19 +2178,19 @@
           <t>ถ้าออกมาเป็น in_progress ต้องได้ grade: null และอีเมลต้องไม่มี Grade ติดไปด้วย ส่วนการสรุปผลที่ล้มเหลวก็ต้องไม่คืนและไม่ส่ง Grade และทั้งสองฝั่งต้องได้พฤติกรรมเดียวกันเพราะใช้ service ร่วมกัน</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>ยังไม่ได้รัน
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
 หลักฐาน: verdict — กรณีผู้ดูแลได้ Grade เป็น null ตอนส่งกลับไปแก้ไข และการตรวจ Grade ที่เข้มขึ้นในกรณี finished
-ผลที่บันทึกไว้: ยังไม่ commit</t>
+ผลที่บันทึกไว้: 30/30 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>011-FR-4
-สัญญาเดิมทั้งหมดต้องไม่เปลี่ยน</t>
+สัญญาเดิมทั้งหมดต้องไม่เปลี่ยน  ✓ รันแล้ว</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -2003,19 +2198,19 @@
           <t>ไม่เพิ่ม ไม่ลบ ไม่เปลี่ยนชื่อ endpoint ไม่แตะสิทธิ์ ไม่แตะ status code สูตรคะแนน การแยกตามหมวด เกณฑ์ Grade และเงื่อนไขข้อ special เหมือนเดิม และ grade ยังเป็น nullable ตามเดิม</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>ยังไม่ได้รัน
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
 หลักฐาน: score.test.ts — รับ Grade เป็น null ได้, รับ Grade ครบทั้งสี่ค่า และปฏิเสธค่า "platinum"
-ผลที่บันทึกไว้: ยังไม่ commit</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+ผลที่บันทึกไว้: 27/27 · ชุดทดสอบเต็ม ณ run นั้น 537/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>011-FR-5
-ต้องมีเทสต์ถดถอยรองรับ</t>
+ต้องมีเทสต์ถดถอยรองรับ  ✓ รันแล้ว</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -2023,11 +2218,11 @@
           <t>ครอบคลุมทั้งสามสถานะ การเรียงล็อกเมื่อมีหลายแถว ทั้งรายงานโรงงานและรายการเจ้าหน้าที่ ความเท่าเทียมของการสรุปผลทั้งสองฝั่ง และต้องตรวจทั้งด้านบวก (finished ได้ Grade) และด้านลบ (ไม่ finished ต้องไม่มี Grade)</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>ยังไม่ได้รัน
-หลักฐาน: สี่แถวข้างบนคือความครอบคลุมที่ข้อกำหนดนี้ต้องการ (G-5)
-ผลที่บันทึกไว้: ยังไม่ commit — bolt 024 ยังไม่มีรายงานผลการทดสอบ</t>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: สี่แถวข้างบนรวมกันคือความครอบคลุมที่ข้อกำหนดนี้ต้องการ หมายเหตุ: bolt 024 ยังไม่มีไฟล์ ddd-03-test-report.md ของตัวเอง หลักฐานที่ใช้คือชุดทดสอบเต็มของ run 009/010
+ผลที่บันทึกไว้: ชุดทดสอบเต็ม ณ run นั้น 537/0 — ปิดช่องว่าง G-5</t>
         </is>
       </c>
     </row>
@@ -2035,4 +2230,249 @@
   <autoFilter ref="A4:C9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Intent SCF — Score-Change Finality (ADR-0012)  ★ ใหม่</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>intent ล่าสุด ปิดงาน 25 ส.ค. 2569 ระดับความเร่งด่วน urgent ทำผ่าน FIRE 6 work item (run 005–010) แก้ปัญหาที่ production ทำลายหลักฐานของโรงงานทุกครั้งที่ผู้ตรวจแก้คะแนน มาตั้งแต่ 7 ก.ค. 2569 แทนที่ ADR-0006 ทั้งฉบับ และแทนที่ ADR-0004 บางส่วน</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>requirement</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>ผลการทดสอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="108" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>SCF-1
+การแก้คะแนนเป็นคำวินิจฉัยที่สิ้นสุด  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>change_score บันทึกเป็น recommended พร้อมเก็บ verdictChoice และคำอธิบายไว้ มีแค่ hard reject ที่ได้ rejected ทั้งหมดนี้อยู่ในนิพจน์เดียวที่ evaluator-review.ts:315 และตามมาด้วยผลข้างเคียงทุกอย่างที่เคยผูกกับ rejected ทั้งการลบไฟล์ สถานะ Cover สิทธิ์ต่อรอง และคะแนนที่เข้า Grade
+หมายเหตุ: เดิมออกแบบให้ตรวจหลักฐานตอนบันทึก (400 ถ้าไฟล์ไม่รองรับคะแนนใหม่) แต่ human กลับคำ 24 ส.ค. 2569 เพราะการปฏิเสธจะเหลือทางเดียวคือ hard reject ซึ่งลบหลักฐานของโรงงาน แย่กว่าการเชื่อคำวินิจฉัยของผู้ตรวจ</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: save — change_score → recommended, reject → rejected + null, approve ไม่เปลี่ยน, no-op ยัง 400, กติกาแก้ไขของ recommended คุมการแก้คะแนนด้วย, และ describe “A change_score is never evidence-checked” ยืนยันว่าไม่มีการตรวจไฟล์ทั้งขาขึ้นและขาลง
+ผลที่บันทึกไว้: 26/26 (โต 19 → 26), run 005, 24 ส.ค. 2569 · ชุดเต็ม 518/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="108" customHeight="1">
+      <c r="A6" s="21" t="inlineStr">
+        <is>
+          <t>SCF-2
+การสรุปผลตัดสินคะแนนและเก็บหลักฐานไว้  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>ตอนสรุปผล ระบบเขียน verdictChoice ลง answers.selectedChoice ในทรานแซกชันเดียวกับ การเลื่อน recommended → finished เพื่อให้ Grade คิดจากคะแนนที่แก้แล้ว Cover ที่มีแต่ approve กับ change-score ไปถึง finished ได้ในรอบเดียว ไม่มีการเด้งกลับ และไฟล์ของข้อที่ถูกแก้คะแนนต้องยังอยู่ทั้งใน MinIO และในฐานข้อมูล
+แถวรูปแบบเก่าที่บันทึกไว้ก่อนเปลี่ยนกติกา (rejected + verdict_choice ไม่ null) ต้องถูกจัดเป็นการแก้คะแนนโดยอัตโนมัติ ไม่ต้อง backfill</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — ชุดที่ลบเหลือแค่ hard reject, Cover จบในรอบเดียว, selectedChoice := verdictChoice, Grade เปลี่ยนตามคะแนนที่แก้, แถวรูปแบบเก่าจบงานได้เอง, hard reject ไม่เปลี่ยนพฤติกรรม, แถวเลื่อนสถานะพา verdictChoice ไปด้วย และการสรุปผลซ้ำไม่สร้างล็อกซ้ำ
+ผลที่บันทึกไว้: 23/23 (โต 17 → 23), run 006, 24 ส.ค. 2569 · ชุดเต็ม 524/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="21" t="inlineStr">
+        <is>
+          <t>SCF-3
+เลิกใช้เส้นทางต่อรองสำหรับการแก้คะแนน  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>accept และ redo บนคำตอบที่ถูกแก้คะแนนต้องตอบ 400 พร้อมข้อความที่บอกเหตุผลชัดเจน ครอบคลุมทั้งรูปแบบใหม่ (recommended) และรูปแบบเก่า (rejected + verdictChoice) ส่วน hard reject ยังใช้เส้นทางเดิมทุกอย่าง และคำอธิบายของผู้ตรวจต้องรอดไปถึงตอนสรุปผล เพื่อให้โรงงานรู้เหตุผลของคะแนนที่เปลี่ยน</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: answer.integration — describe “negotiate — a settled score change admits no factory response” 4 กรณี ; verdict — กรณีแถวเลื่อนสถานะขยายให้ตรวจ description ด้วย ก่อนหน้านี้เส้นทาง negotiate ไม่เคยมีเทสต์เลยแม้แต่กรณีเดียว
+ผลที่บันทึกไว้: 9/9, run 007, 24 ส.ค. 2569 · ชุดเต็ม 528/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="21" t="inlineStr">
+        <is>
+          <t>SCF-4
+การอ่านข้อมูลกลับหลังสรุปผล  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>เดิมตั้งใจให้อีเมล finished ไล่รายการข้อที่ถูกแก้คะแนน แต่ human ตัดสินใจ 24 ส.ค. 2569 ว่าไม่ต้องแก้อีเมล เปลี่ยนเป็นพิสูจน์ว่าเส้นทางอ่านของโรงงานพาข้อมูลที่แก้แล้วกลับมาได้จริง คือคืน status finished, verdictChoice ที่ผู้ตรวจตั้ง, เหตุผลภาษาไทย และ selectedChoice ที่เป็นค่าที่แก้แล้ว ส่วนข้อที่ไม่ถูกแตะจะมี verdictChoice เป็น null ซึ่งเป็นตัวที่หน้าจอใช้แยกความต่าง</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: answer.integration — describe “getAnswerByFactoryId — a settled correction after finalize” 2 กรณี รัน finalize จริงแล้วอ่านกลับผ่าน service ของฝั่งโรงงาน เป็นการเชื่อมฝั่งผู้ประเมินกับฝั่งโรงงานแบบครบวงจรครั้งแรก run นี้ไม่ได้เขียนโค้ด production เลย
+ผลที่บันทึกไว้: 9/9, run 008, 24 ส.ค. 2569 · ชุดเต็ม 530/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>SCF-5
+hard reject ลบใบรับรองมาตรฐานด้วย  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>เมื่อ hard reject คำถามที่อ้างอิงมาตรฐาน ให้ลบใบรับรองมาตรฐานทุกใบที่คำถามข้อนั้นระบุ และโรงงานแจ้งไว้ พร้อมล้างทั้งค่า boolean และ url บนแถวการลงทะเบียน ใบที่ใช้ร่วมกันหลายคำถามต้องถูกลบครั้งเดียว ใบที่โรงงานไม่ได้แจ้งต้องไม่ถูกแตะ ส่วนคำตอบข้ออื่นที่เคยได้คะแนนจากใบที่ถูกลบ ถ้ายังไม่ finished ให้กลับไป in_review แต่ถ้า finished แล้วต้องไม่ถูกแตะ และการแก้คะแนนต้องไม่ลบอะไรเลย</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: verdict — 7 กรณีใหม่ใน 2 describe ครอบคลุมการลบตามที่แจ้งไว้ ใบที่ใช้ร่วมกัน การล้างค่าบนแถวการลงทะเบียน คำตอบข้างเคียงทั้งที่ finished แล้วและยังไม่ และการยืนยันว่าการแก้คะแนนไม่ลบใบรับรองเลย
+ผลที่บันทึกไว้: 30/30 (โต 23 → 30), run 009, 25 ส.ค. 2569 · ชุดเต็ม 537/0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="80" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>SCF-6
+บันทึกการกลับคำและปรับเอกสารโดเมน  ★ ใหม่</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>ออก ADR-0012 ที่ระบุชัดว่าแทนที่ ADR-0006 ทั้งฉบับ และแทนที่ ADR-0004 บางส่วน พร้อมคืนข้อกำหนดเรื่องการเก็บไฟล์ของ ADR-0005 ใส่หมายเหตุ superseded-by บน ADR ทั้งสองฉบับ โดยไม่แก้เหตุผลเดิม บันทึกเงื่อนไข verdict_choice IS NULL ไว้เป็นสัญญาที่ต้องรักษา พร้อมคำเตือนว่าอย่าลดรูปเหลือการเช็ก status อย่างเดียว และปรับ CONTEXT.md ทุกหัวข้อที่เกี่ยวข้อง รวมถึงแผนภาพและตารางเส้นทาง API</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: เป็น run ที่ทำเอกสารอย่างเดียว ไม่มีเทสต์ใหม่และไม่จำเป็นต้องมี รันชุดทดสอบเต็มเพื่อยืนยันว่าไม่มีพฤติกรรมไหนเปลี่ยน ทุกจุดที่ ADR อ้างถึงในโค้ดถูกเปิดตรวจกับ source จริงก่อนเขียน และการ grep หาข้อความเก่ายังเจอจุดตกหล่นอีก 2 แห่งที่แผนไม่ได้ระบุไว้
+ผลที่บันทึกไว้: 537/0, run 010, 25 ส.ค. 2569 (ไม่แตะพฤติกรรม)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:C10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="82" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Intent AFE — Admin Factory List Exposes Account Email  ⚑ นอกขอบเขตโมดูลการประเมิน</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>⚑ intent ล่าสุด (run 011, ปิดงาน 26 ส.ค. 2569) แต่เป็นงานของโดเมนโรงงาน ไม่ใช่โมดูลการประเมิน จึงแยกไว้เป็นชีตต่างหากและไม่นับรวมในยอด 43 ข้อของโมดูล บันทึกไว้เพื่อให้ตารางตามงาน FIRE ทัน สถานะโค้ดตอนนี้: แก้แล้วแต่ยังไม่ commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>requirement</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>ผลการทดสอบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="136" customHeight="1">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>AFE-1
+เพิ่ม email ของบัญชีในรายการโรงงานฝั่งผู้ดูแล  ⚑ นอกขอบเขต</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>GET /twhp/api/admins/factories คืนฟิลด์ email ของทุกรายการในหน้า โดยเอาค่ามาจาก accounts.email ของบัญชีโรงงานนั้นเอง (join ที่ factories.accountId = accounts.id) และประกาศไว้ใน response schema เพื่อให้ขึ้นในเอกสาร OpenAPI ด้วย
+ข้อจำกัดสำคัญ: เพิ่มเฉพาะ projection ของฝั่งผู้ดูแลเท่านั้น ห้ามแตะ factoryListColumns ที่ใช้ร่วมกันทั้งสามรายการ เพราะจะทำให้ฝั่งเจ้าหน้าที่จังหวัดและผู้ประเมินเห็น email ไปด้วย และต้องเป็น accounts.email ไม่ใช่ factories.safetyOfficerEmail ซึ่งคนละความหมาย ส่วน pagination การเรียง และตัวกรอง validated / enrolled ต้องไม่เปลี่ยน</t>
+        </is>
+      </c>
+      <c r="C5" s="20" t="inlineStr">
+        <is>
+          <t>ยืนยันแล้ว
+หลักฐาน: factory-pagination.integration — Story 011 รวม 9 กรณี แบ่งเป็นแบบต่อฐานข้อมูลจริง 6 กรณี (ทุกรายการมี email, จับคู่บัญชีถูกตัว, email กับ username มาจากบัญชีเดียวกัน, ฝั่งผู้ประเมินไม่มี email, ฝั่งจังหวัดไม่มี email, pagination ไม่เพี้ยน) และแบบอ่าน schema ของ route อีก 3 กรณี มีการทำ negative control ด้วย คือย้อนการแก้ทีละครึ่งแล้วรันใหม่ เพื่อพิสูจน์ว่าทั้งสองจุดจำเป็นจริง และเปิด JUnit report ยืนยันว่ากรณีที่ต่อฐานข้อมูลรันจริง ไม่ได้ถูก describeDb ข้ามไปเงียบ ๆ
+ผลที่บันทึกไว้: 9/9 · ชุดทดสอบเต็มบน dev 392/0 (โต 383 → 392), run 011, 26 ส.ค. 2569</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:C5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>